<commit_message>
top 9 feature importance
</commit_message>
<xml_diff>
--- a/Sentinel_Mean_Regression_Results.xlsx
+++ b/Sentinel_Mean_Regression_Results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D136"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,7 +434,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Coefficient</t>
+          <t>B1_Coefficient</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>B0_Y_Intercept</t>
         </is>
       </c>
     </row>
@@ -453,6 +458,9 @@
       <c r="D2" t="n">
         <v>-29.00517309898451</v>
       </c>
+      <c r="E2" t="n">
+        <v>37.39284534927025</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -469,6 +477,9 @@
       <c r="D3" t="n">
         <v>-52.19075053280852</v>
       </c>
+      <c r="E3" t="n">
+        <v>8.119935024007077</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -485,6 +496,9 @@
       <c r="D4" t="n">
         <v>22.37143264238413</v>
       </c>
+      <c r="E4" t="n">
+        <v>-14.42082371995382</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -501,6 +515,9 @@
       <c r="D5" t="n">
         <v>-14.42155059244365</v>
       </c>
+      <c r="E5" t="n">
+        <v>27.44949905412884</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -517,6 +534,9 @@
       <c r="D6" t="n">
         <v>-32.63354986247916</v>
       </c>
+      <c r="E6" t="n">
+        <v>12.47398284335752</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -533,6 +553,9 @@
       <c r="D7" t="n">
         <v>-35.88818380533679</v>
       </c>
+      <c r="E7" t="n">
+        <v>18.02003728786612</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -549,6 +572,9 @@
       <c r="D8" t="n">
         <v>25.19257651264596</v>
       </c>
+      <c r="E8" t="n">
+        <v>-6.405527102190123</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -565,6 +591,9 @@
       <c r="D9" t="n">
         <v>-10.32013256688555</v>
       </c>
+      <c r="E9" t="n">
+        <v>27.10436230955205</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,6 +610,9 @@
       <c r="D10" t="n">
         <v>16.21393103306397</v>
       </c>
+      <c r="E10" t="n">
+        <v>-4.294955324567304</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -597,6 +629,9 @@
       <c r="D11" t="n">
         <v>-17.93164323626965</v>
       </c>
+      <c r="E11" t="n">
+        <v>16.37456318952108</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -613,6 +648,9 @@
       <c r="D12" t="n">
         <v>-15.14169228983445</v>
       </c>
+      <c r="E12" t="n">
+        <v>16.11785972806552</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -629,6 +667,9 @@
       <c r="D13" t="n">
         <v>-14.2986348714893</v>
       </c>
+      <c r="E13" t="n">
+        <v>29.3352358846582</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -645,6 +686,9 @@
       <c r="D14" t="n">
         <v>-32.14186127065256</v>
       </c>
+      <c r="E14" t="n">
+        <v>14.91912819075231</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -661,6 +705,9 @@
       <c r="D15" t="n">
         <v>-3.535816676846845</v>
       </c>
+      <c r="E15" t="n">
+        <v>18.24741756957153</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -677,6 +724,9 @@
       <c r="D16" t="n">
         <v>9.651135797301045</v>
       </c>
+      <c r="E16" t="n">
+        <v>5.892584900464014</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -693,6 +743,9 @@
       <c r="D17" t="n">
         <v>17.63255637222903</v>
       </c>
+      <c r="E17" t="n">
+        <v>-2.832328811346514</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -709,6 +762,9 @@
       <c r="D18" t="n">
         <v>-12.5625000688253</v>
       </c>
+      <c r="E18" t="n">
+        <v>16.7805749266264</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -725,6 +781,9 @@
       <c r="D19" t="n">
         <v>9.610048359697961</v>
       </c>
+      <c r="E19" t="n">
+        <v>6.25999037336157</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -741,6 +800,9 @@
       <c r="D20" t="n">
         <v>9.387822246437924</v>
       </c>
+      <c r="E20" t="n">
+        <v>7.567982467199732</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -757,6 +819,9 @@
       <c r="D21" t="n">
         <v>-10.9281260367274</v>
       </c>
+      <c r="E21" t="n">
+        <v>16.43589460608845</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -773,6 +838,9 @@
       <c r="D22" t="n">
         <v>7.834196864589207</v>
       </c>
+      <c r="E22" t="n">
+        <v>6.123736213530728</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -789,6 +857,9 @@
       <c r="D23" t="n">
         <v>-12.65411902938489</v>
       </c>
+      <c r="E23" t="n">
+        <v>14.05052006652724</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -805,6 +876,9 @@
       <c r="D24" t="n">
         <v>8.696253403459128</v>
       </c>
+      <c r="E24" t="n">
+        <v>8.125241894449227</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -821,6 +895,9 @@
       <c r="D25" t="n">
         <v>-10.19727867607763</v>
       </c>
+      <c r="E25" t="n">
+        <v>15.53994283359393</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -837,6 +914,9 @@
       <c r="D26" t="n">
         <v>7.897158335256194</v>
       </c>
+      <c r="E26" t="n">
+        <v>6.435368015269376</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -853,6 +933,9 @@
       <c r="D27" t="n">
         <v>-9.559654534023368</v>
       </c>
+      <c r="E27" t="n">
+        <v>14.71505318320968</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -869,6 +952,9 @@
       <c r="D28" t="n">
         <v>8.342667732080294</v>
       </c>
+      <c r="E28" t="n">
+        <v>9.625212737050525</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -885,6 +971,9 @@
       <c r="D29" t="n">
         <v>-13.52334242383457</v>
       </c>
+      <c r="E29" t="n">
+        <v>22.85834820220455</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -901,6 +990,9 @@
       <c r="D30" t="n">
         <v>-10.68231187628779</v>
       </c>
+      <c r="E30" t="n">
+        <v>14.05852295892381</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -917,6 +1009,9 @@
       <c r="D31" t="n">
         <v>17.65787041837072</v>
       </c>
+      <c r="E31" t="n">
+        <v>9.978734306497042</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -933,6 +1028,9 @@
       <c r="D32" t="n">
         <v>-7.434072432146733</v>
       </c>
+      <c r="E32" t="n">
+        <v>15.57269105193213</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -949,6 +1047,9 @@
       <c r="D33" t="n">
         <v>-7.672453997752628</v>
       </c>
+      <c r="E33" t="n">
+        <v>16.50479374744884</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -965,6 +1066,9 @@
       <c r="D34" t="n">
         <v>8.106520235091757</v>
       </c>
+      <c r="E34" t="n">
+        <v>10.23024117554199</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -981,6 +1085,9 @@
       <c r="D35" t="n">
         <v>-1.492972690674861</v>
       </c>
+      <c r="E35" t="n">
+        <v>15.72913795288743</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -997,6 +1104,9 @@
       <c r="D36" t="n">
         <v>5.965589635673762</v>
       </c>
+      <c r="E36" t="n">
+        <v>9.711065395051474</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1013,6 +1123,9 @@
       <c r="D37" t="n">
         <v>5.867278858977642</v>
       </c>
+      <c r="E37" t="n">
+        <v>8.545069329683725</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1029,6 +1142,9 @@
       <c r="D38" t="n">
         <v>6.343352697230328</v>
       </c>
+      <c r="E38" t="n">
+        <v>4.977901697866796</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1045,6 +1161,9 @@
       <c r="D39" t="n">
         <v>-5.196776054436859</v>
       </c>
+      <c r="E39" t="n">
+        <v>20.71781598873045</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1061,6 +1180,9 @@
       <c r="D40" t="n">
         <v>7.268211277133064</v>
       </c>
+      <c r="E40" t="n">
+        <v>3.296420078780299</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1077,6 +1199,9 @@
       <c r="D41" t="n">
         <v>1.197192065832873</v>
       </c>
+      <c r="E41" t="n">
+        <v>9.721472344036355</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1093,6 +1218,9 @@
       <c r="D42" t="n">
         <v>19.06601425707996</v>
       </c>
+      <c r="E42" t="n">
+        <v>10.41557457583378</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1109,6 +1237,9 @@
       <c r="D43" t="n">
         <v>7.247413063853084</v>
       </c>
+      <c r="E43" t="n">
+        <v>9.633445850892489</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1125,6 +1256,9 @@
       <c r="D44" t="n">
         <v>-11.35128209442091</v>
       </c>
+      <c r="E44" t="n">
+        <v>21.71010600938428</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1141,6 +1275,9 @@
       <c r="D45" t="n">
         <v>6.020132554221383</v>
       </c>
+      <c r="E45" t="n">
+        <v>8.929331028083897</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1157,6 +1294,9 @@
       <c r="D46" t="n">
         <v>-7.747715500903948</v>
       </c>
+      <c r="E46" t="n">
+        <v>15.65217652356689</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1173,6 +1313,9 @@
       <c r="D47" t="n">
         <v>14.02032843874647</v>
       </c>
+      <c r="E47" t="n">
+        <v>11.43609987736121</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1189,6 +1332,9 @@
       <c r="D48" t="n">
         <v>5.714989076276411</v>
       </c>
+      <c r="E48" t="n">
+        <v>10.31716584952089</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1205,6 +1351,9 @@
       <c r="D49" t="n">
         <v>-16.17201066124651</v>
       </c>
+      <c r="E49" t="n">
+        <v>15.95160125083719</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1221,6 +1370,9 @@
       <c r="D50" t="n">
         <v>-6.729244100333486</v>
       </c>
+      <c r="E50" t="n">
+        <v>16.51772500964177</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1237,6 +1389,9 @@
       <c r="D51" t="n">
         <v>6.289683164590596</v>
       </c>
+      <c r="E51" t="n">
+        <v>9.590259983361689</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1253,6 +1408,9 @@
       <c r="D52" t="n">
         <v>7.382734185146549</v>
       </c>
+      <c r="E52" t="n">
+        <v>10.10721944507333</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1269,6 +1427,9 @@
       <c r="D53" t="n">
         <v>11.20891805856816</v>
       </c>
+      <c r="E53" t="n">
+        <v>5.107320755008193</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1285,6 +1446,9 @@
       <c r="D54" t="n">
         <v>9.288022934112885</v>
       </c>
+      <c r="E54" t="n">
+        <v>2.459760989586178</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1301,6 +1465,9 @@
       <c r="D55" t="n">
         <v>2.428094989430217</v>
       </c>
+      <c r="E55" t="n">
+        <v>8.86361538156469</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1317,6 +1484,9 @@
       <c r="D56" t="n">
         <v>4.918757341526837</v>
       </c>
+      <c r="E56" t="n">
+        <v>9.812255684687017</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1333,6 +1503,9 @@
       <c r="D57" t="n">
         <v>-5.827687824893947</v>
       </c>
+      <c r="E57" t="n">
+        <v>15.39900327086898</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1349,6 +1522,9 @@
       <c r="D58" t="n">
         <v>-2.692674765907035</v>
       </c>
+      <c r="E58" t="n">
+        <v>15.97437595564083</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1365,6 +1541,9 @@
       <c r="D59" t="n">
         <v>7.340902643366459</v>
       </c>
+      <c r="E59" t="n">
+        <v>9.652155727056494</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1381,6 +1560,9 @@
       <c r="D60" t="n">
         <v>0.4725889340464339</v>
       </c>
+      <c r="E60" t="n">
+        <v>10.91896208906145</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1397,6 +1579,9 @@
       <c r="D61" t="n">
         <v>-0.7725800039809205</v>
       </c>
+      <c r="E61" t="n">
+        <v>14.65544737426659</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1413,6 +1598,9 @@
       <c r="D62" t="n">
         <v>15.69160302773643</v>
       </c>
+      <c r="E62" t="n">
+        <v>11.88775117016855</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1429,6 +1617,9 @@
       <c r="D63" t="n">
         <v>-5.067251098403565</v>
       </c>
+      <c r="E63" t="n">
+        <v>16.80975272047608</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1445,6 +1636,9 @@
       <c r="D64" t="n">
         <v>2.088360104142621</v>
       </c>
+      <c r="E64" t="n">
+        <v>8.533973143259905</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1461,6 +1655,9 @@
       <c r="D65" t="n">
         <v>1.034916038811262</v>
       </c>
+      <c r="E65" t="n">
+        <v>10.13282236569022</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1477,6 +1674,9 @@
       <c r="D66" t="n">
         <v>-5.968022801977399</v>
       </c>
+      <c r="E66" t="n">
+        <v>14.48646536129424</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1493,6 +1693,9 @@
       <c r="D67" t="n">
         <v>-6.051760031028159</v>
       </c>
+      <c r="E67" t="n">
+        <v>15.25198755056032</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1509,6 +1712,9 @@
       <c r="D68" t="n">
         <v>4.232825218130526</v>
       </c>
+      <c r="E68" t="n">
+        <v>10.11395687225409</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1525,6 +1731,9 @@
       <c r="D69" t="n">
         <v>-5.742083763542584</v>
       </c>
+      <c r="E69" t="n">
+        <v>17.76515559701221</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1541,6 +1750,9 @@
       <c r="D70" t="n">
         <v>8.044063893497585</v>
       </c>
+      <c r="E70" t="n">
+        <v>9.991630407621399</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1557,6 +1769,9 @@
       <c r="D71" t="n">
         <v>4.677048362788116</v>
       </c>
+      <c r="E71" t="n">
+        <v>9.187520558992357</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1573,6 +1788,9 @@
       <c r="D72" t="n">
         <v>-5.479233180743381</v>
       </c>
+      <c r="E72" t="n">
+        <v>14.29615985115621</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1589,6 +1807,9 @@
       <c r="D73" t="n">
         <v>1.650434688162062</v>
       </c>
+      <c r="E73" t="n">
+        <v>11.16493911087986</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1605,6 +1826,9 @@
       <c r="D74" t="n">
         <v>-4.554965305584282</v>
       </c>
+      <c r="E74" t="n">
+        <v>14.49137906132659</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1621,6 +1845,9 @@
       <c r="D75" t="n">
         <v>0.6005051069637291</v>
       </c>
+      <c r="E75" t="n">
+        <v>10.0840778103527</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1637,6 +1864,9 @@
       <c r="D76" t="n">
         <v>0.7543924191782247</v>
       </c>
+      <c r="E76" t="n">
+        <v>11.53036539609761</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1653,6 +1883,9 @@
       <c r="D77" t="n">
         <v>7.179896188683697</v>
       </c>
+      <c r="E77" t="n">
+        <v>10.42339340765559</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1669,6 +1902,9 @@
       <c r="D78" t="n">
         <v>-5.651550847792978</v>
       </c>
+      <c r="E78" t="n">
+        <v>13.54989998491456</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1685,6 +1921,9 @@
       <c r="D79" t="n">
         <v>3.336108855716279</v>
       </c>
+      <c r="E79" t="n">
+        <v>9.687538776871683</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1701,6 +1940,9 @@
       <c r="D80" t="n">
         <v>-3.314928374822759</v>
       </c>
+      <c r="E80" t="n">
+        <v>14.12221368549439</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1717,6 +1959,9 @@
       <c r="D81" t="n">
         <v>1.503339876292806</v>
       </c>
+      <c r="E81" t="n">
+        <v>11.25213570387365</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1733,6 +1978,9 @@
       <c r="D82" t="n">
         <v>1.104027951751813</v>
       </c>
+      <c r="E82" t="n">
+        <v>11.25544888758015</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1749,6 +1997,9 @@
       <c r="D83" t="n">
         <v>0.5006670216251226</v>
       </c>
+      <c r="E83" t="n">
+        <v>11.58353144885234</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1765,6 +2016,9 @@
       <c r="D84" t="n">
         <v>-4.842905309882253</v>
       </c>
+      <c r="E84" t="n">
+        <v>15.02196070959434</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1781,6 +2035,9 @@
       <c r="D85" t="n">
         <v>-0.3202433250008188</v>
       </c>
+      <c r="E85" t="n">
+        <v>13.638045066361</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1797,6 +2054,9 @@
       <c r="D86" t="n">
         <v>-0.3657768294850438</v>
       </c>
+      <c r="E86" t="n">
+        <v>13.8021031105452</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1813,6 +2073,9 @@
       <c r="D87" t="n">
         <v>-4.363355853418612</v>
       </c>
+      <c r="E87" t="n">
+        <v>14.89931352058207</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1829,6 +2092,9 @@
       <c r="D88" t="n">
         <v>0.2957745300043728</v>
       </c>
+      <c r="E88" t="n">
+        <v>10.64052398058849</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1845,6 +2111,9 @@
       <c r="D89" t="n">
         <v>-4.879560491128608</v>
       </c>
+      <c r="E89" t="n">
+        <v>13.02241130768943</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1861,6 +2130,9 @@
       <c r="D90" t="n">
         <v>0.9588466204398332</v>
       </c>
+      <c r="E90" t="n">
+        <v>11.36235156142849</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1877,6 +2149,9 @@
       <c r="D91" t="n">
         <v>4.126396480450954</v>
       </c>
+      <c r="E91" t="n">
+        <v>7.60107447634361</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1893,6 +2168,9 @@
       <c r="D92" t="n">
         <v>2.57392087566757</v>
       </c>
+      <c r="E92" t="n">
+        <v>10.85228482830819</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1909,6 +2187,9 @@
       <c r="D93" t="n">
         <v>-11.28024311332188</v>
       </c>
+      <c r="E93" t="n">
+        <v>11.68796746891157</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1925,6 +2206,9 @@
       <c r="D94" t="n">
         <v>-0.1656157217671643</v>
       </c>
+      <c r="E94" t="n">
+        <v>13.21466066441096</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1941,6 +2225,9 @@
       <c r="D95" t="n">
         <v>-0.5239124523093041</v>
       </c>
+      <c r="E95" t="n">
+        <v>13.50307154546011</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1957,6 +2244,9 @@
       <c r="D96" t="n">
         <v>-6.202865928538541</v>
       </c>
+      <c r="E96" t="n">
+        <v>17.90438407755283</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1973,6 +2263,9 @@
       <c r="D97" t="n">
         <v>-2.482102503116476</v>
       </c>
+      <c r="E97" t="n">
+        <v>12.98649831827161</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1989,6 +2282,9 @@
       <c r="D98" t="n">
         <v>0.2673902668480278</v>
       </c>
+      <c r="E98" t="n">
+        <v>11.51469940036257</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2005,6 +2301,9 @@
       <c r="D99" t="n">
         <v>-2.185495078351455</v>
       </c>
+      <c r="E99" t="n">
+        <v>12.74337228114739</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2021,6 +2320,9 @@
       <c r="D100" t="n">
         <v>1.440380282190264</v>
       </c>
+      <c r="E100" t="n">
+        <v>11.15072573699518</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2037,6 +2339,9 @@
       <c r="D101" t="n">
         <v>0.298652253147675</v>
       </c>
+      <c r="E101" t="n">
+        <v>11.17572540143956</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2053,6 +2358,9 @@
       <c r="D102" t="n">
         <v>2.490844934373027</v>
       </c>
+      <c r="E102" t="n">
+        <v>10.91870391463269</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2069,6 +2377,9 @@
       <c r="D103" t="n">
         <v>0.5395913562673269</v>
       </c>
+      <c r="E103" t="n">
+        <v>10.98016394364024</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2085,6 +2396,9 @@
       <c r="D104" t="n">
         <v>0.3201365424105347</v>
       </c>
+      <c r="E104" t="n">
+        <v>11.17350644126631</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2101,6 +2415,9 @@
       <c r="D105" t="n">
         <v>0.5735362644677283</v>
       </c>
+      <c r="E105" t="n">
+        <v>10.98214485366469</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2117,6 +2434,9 @@
       <c r="D106" t="n">
         <v>-0.3621464979539335</v>
       </c>
+      <c r="E106" t="n">
+        <v>12.77582206177269</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2133,6 +2453,9 @@
       <c r="D107" t="n">
         <v>-0.2203664422641429</v>
       </c>
+      <c r="E107" t="n">
+        <v>12.9424415238163</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2149,6 +2472,9 @@
       <c r="D108" t="n">
         <v>1.780679634048669</v>
       </c>
+      <c r="E108" t="n">
+        <v>9.58591240092791</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2165,6 +2491,9 @@
       <c r="D109" t="n">
         <v>-2.168721365028717</v>
       </c>
+      <c r="E109" t="n">
+        <v>12.57387950633728</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2181,6 +2510,9 @@
       <c r="D110" t="n">
         <v>0.1085689604384635</v>
       </c>
+      <c r="E110" t="n">
+        <v>11.6821242435173</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2197,6 +2529,9 @@
       <c r="D111" t="n">
         <v>-1.681347006162627</v>
       </c>
+      <c r="E111" t="n">
+        <v>12.34737332273673</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2213,6 +2548,9 @@
       <c r="D112" t="n">
         <v>-4.415068002057682</v>
       </c>
+      <c r="E112" t="n">
+        <v>11.3811806838462</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2229,6 +2567,9 @@
       <c r="D113" t="n">
         <v>-0.1870821939170784</v>
       </c>
+      <c r="E113" t="n">
+        <v>12.57797301900813</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2245,6 +2586,9 @@
       <c r="D114" t="n">
         <v>-2.459525790062898</v>
       </c>
+      <c r="E114" t="n">
+        <v>14.21150201160853</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2261,6 +2605,9 @@
       <c r="D115" t="n">
         <v>0.1139529490995302</v>
       </c>
+      <c r="E115" t="n">
+        <v>11.77856978297078</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2277,6 +2624,9 @@
       <c r="D116" t="n">
         <v>0.256481546468785</v>
       </c>
+      <c r="E116" t="n">
+        <v>11.47097862510817</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2293,6 +2643,9 @@
       <c r="D117" t="n">
         <v>-2.317124417992252</v>
       </c>
+      <c r="E117" t="n">
+        <v>13.78202250949648</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2309,6 +2662,9 @@
       <c r="D118" t="n">
         <v>-1.177436416661644</v>
       </c>
+      <c r="E118" t="n">
+        <v>12.50986298192138</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2325,6 +2681,9 @@
       <c r="D119" t="n">
         <v>1.406216028334585</v>
       </c>
+      <c r="E119" t="n">
+        <v>11.26365051938819</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2341,6 +2700,9 @@
       <c r="D120" t="n">
         <v>1.999554619527542</v>
       </c>
+      <c r="E120" t="n">
+        <v>10.6165096281592</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2357,6 +2719,9 @@
       <c r="D121" t="n">
         <v>-0.1618487184751147</v>
       </c>
+      <c r="E121" t="n">
+        <v>12.39129020030294</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2373,6 +2738,9 @@
       <c r="D122" t="n">
         <v>0.2173424749587569</v>
       </c>
+      <c r="E122" t="n">
+        <v>11.70377808444509</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2389,6 +2757,9 @@
       <c r="D123" t="n">
         <v>2.389418862078953</v>
       </c>
+      <c r="E123" t="n">
+        <v>11.88619125016587</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2405,6 +2776,9 @@
       <c r="D124" t="n">
         <v>0.3009537336131254</v>
       </c>
+      <c r="E124" t="n">
+        <v>11.59281437408086</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2421,6 +2795,9 @@
       <c r="D125" t="n">
         <v>-2.270003509723648</v>
       </c>
+      <c r="E125" t="n">
+        <v>12.44180350261952</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2437,6 +2814,9 @@
       <c r="D126" t="n">
         <v>-0.8130678827282125</v>
       </c>
+      <c r="E126" t="n">
+        <v>12.39229499157945</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2453,6 +2833,9 @@
       <c r="D127" t="n">
         <v>0.7669824807835806</v>
       </c>
+      <c r="E127" t="n">
+        <v>11.83685121387674</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2469,6 +2852,9 @@
       <c r="D128" t="n">
         <v>0.09683796906673942</v>
       </c>
+      <c r="E128" t="n">
+        <v>11.80607721208711</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2485,6 +2871,9 @@
       <c r="D129" t="n">
         <v>-0.5418950144916841</v>
       </c>
+      <c r="E129" t="n">
+        <v>12.837077825129</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2501,6 +2890,9 @@
       <c r="D130" t="n">
         <v>-0.1131580922898834</v>
       </c>
+      <c r="E130" t="n">
+        <v>12.24714981606565</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2517,6 +2909,9 @@
       <c r="D131" t="n">
         <v>-0.4140638735063531</v>
       </c>
+      <c r="E131" t="n">
+        <v>12.23361240077432</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2533,6 +2928,9 @@
       <c r="D132" t="n">
         <v>0.08684638609911977</v>
       </c>
+      <c r="E132" t="n">
+        <v>11.9081542837784</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2549,6 +2947,9 @@
       <c r="D133" t="n">
         <v>-0.03381739322492183</v>
       </c>
+      <c r="E133" t="n">
+        <v>12.16185070444304</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2565,6 +2966,9 @@
       <c r="D134" t="n">
         <v>-0.2052333696215087</v>
       </c>
+      <c r="E134" t="n">
+        <v>12.30970835251111</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2581,6 +2985,9 @@
       <c r="D135" t="n">
         <v>0.2702322089939306</v>
       </c>
+      <c r="E135" t="n">
+        <v>11.99259681424236</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2596,6 +3003,9 @@
       </c>
       <c r="D136" t="n">
         <v>-0.1733348043080185</v>
+      </c>
+      <c r="E136" t="n">
+        <v>12.10737589598763</v>
       </c>
     </row>
   </sheetData>

</xml_diff>